<commit_message>
Full sync latest POSB dashboard and reports
</commit_message>
<xml_diff>
--- a/Gudivada_Net_Accounts_Latest.xlsx
+++ b/Gudivada_Net_Accounts_Latest.xlsx
@@ -716,52 +716,52 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Bhushanagulla B.O</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>164</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>146</v>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H5" s="10" t="n">
-        <v>97.33333333333334</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>4</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Bollapadu B.O</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Dosapadu B.O</t>
+          <t>Bhushanagulla B.O</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -775,26 +775,26 @@
         <v>150</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>92.66666666666666</v>
+        <v>97.33333333333334</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Koyyagurapadu B.O</t>
+          <t>Dosapadu B.O</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
@@ -808,26 +808,26 @@
         <v>150</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>91.33333333333333</v>
+        <v>92.66666666666666</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Vemanda B.O</t>
+          <t>Koyyagurapadu B.O</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -841,26 +841,26 @@
         <v>150</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>88.66666666666667</v>
+        <v>91.33333333333333</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Bokinala B.O</t>
+          <t>Vemanda B.O</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
@@ -874,26 +874,26 @@
         <v>150</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>85.33333333333334</v>
+        <v>88.66666666666667</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Bollapadu B.O</t>
+          <t>Bokinala B.O</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>150</v>
+        <v>192</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
@@ -907,26 +907,26 @@
         <v>150</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>83.33333333333334</v>
+        <v>85.33333333333334</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Unikili B.O</t>
+          <t>Tummalapalli B.O</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
@@ -940,92 +940,92 @@
         <v>150</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>82</v>
+        <v>85.33333333333334</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
+          <t>Unikili B.O</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>123</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
           <t>Komatigunta Lock B.O</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B13" s="8" t="n">
         <v>191</v>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>69</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>122</v>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>81.33333333333333</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Pedapalaparru B.O</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>137</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>118</v>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>150</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>78.66666666666666</v>
+      <c r="C13" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>121</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>80.66666666666666</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Guruvindagunta B.O</t>
+          <t>Pedapalaparru B.O</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
@@ -1039,26 +1039,26 @@
         <v>150</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>75.33333333333333</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Chowtapalli B.O</t>
+          <t>Moparru B.O</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>171</v>
+        <v>133</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
@@ -1072,26 +1072,26 @@
         <v>150</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Moparru B.O</t>
+          <t>Guruvindagunta B.O</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
@@ -1105,26 +1105,26 @@
         <v>150</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>72.66666666666667</v>
+        <v>75.33333333333333</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Kanukollu B.O</t>
+          <t>Chowtapalli B.O</t>
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="D17" s="14" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
@@ -1138,26 +1138,26 @@
         <v>150</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Tativarru B.O</t>
+          <t>Lingavaram B.O</t>
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D18" s="14" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
@@ -1171,23 +1171,23 @@
         <v>150</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Valivarthipadu B.O</t>
+          <t>Kanukollu B.O</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>108</v>
@@ -1213,17 +1213,17 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Gunnanapudi B.O</t>
+          <t>Tativarru B.O</t>
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D20" s="14" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
@@ -1237,26 +1237,26 @@
         <v>150</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>70.66666666666667</v>
+        <v>72</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Lingavaram B.O</t>
+          <t>Valivarthipadu B.O</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D21" s="14" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
@@ -1270,26 +1270,26 @@
         <v>150</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Velinuthala B.O</t>
+          <t>Gunnanapudi B.O</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D22" s="14" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
@@ -1303,26 +1303,26 @@
         <v>150</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>67.33333333333333</v>
+        <v>70.66666666666667</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Gandhi Asramam B.O</t>
+          <t>Velinuthala B.O</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>107</v>
+        <v>154</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="D23" s="14" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
@@ -1336,23 +1336,23 @@
         <v>150</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>65.33333333333333</v>
+        <v>67.33333333333333</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Nandamuru B.O</t>
+          <t>Gandhi Asramam B.O</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>198</v>
+        <v>107</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="D24" s="14" t="n">
         <v>98</v>
@@ -1378,17 +1378,17 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Garapadu B.O</t>
+          <t>Nandamuru B.O</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>112</v>
+        <v>198</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D25" s="14" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
@@ -1402,26 +1402,26 @@
         <v>150</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>64.66666666666666</v>
+        <v>65.33333333333333</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Putlacheruvu B.O</t>
+          <t>Garapadu B.O</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="D26" s="14" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
@@ -1435,26 +1435,26 @@
         <v>150</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>64</v>
+        <v>64.66666666666666</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>Nandigamalanka B.O</t>
+          <t>Putlacheruvu B.O</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>104</v>
+        <v>137</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
@@ -1468,26 +1468,26 @@
         <v>150</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Ingilipakalanka B.O</t>
+          <t>Nandigamalanka B.O</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
@@ -1501,23 +1501,23 @@
         <v>150</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>59.33333333333334</v>
+        <v>62</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>Vadali B.O</t>
+          <t>Ingilipakalanka B.O</t>
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D29" s="14" t="n">
         <v>89</v>
@@ -1543,17 +1543,17 @@
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Bommuluru B.O</t>
+          <t>Vadali B.O</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>156</v>
+        <v>126</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
@@ -1567,26 +1567,26 @@
         <v>150</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>58.66666666666666</v>
+        <v>59.33333333333334</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Tummalapalli B.O</t>
+          <t>Bommuluru B.O</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>128</v>
+        <v>156</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
@@ -1600,10 +1600,10 @@
         <v>150</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>56.00000000000001</v>
+        <v>58.66666666666666</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32">
@@ -1613,13 +1613,13 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>16</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
@@ -1633,10 +1633,10 @@
         <v>150</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>55.33333333333334</v>
+        <v>57.33333333333334</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33">
@@ -1811,13 +1811,13 @@
         </is>
       </c>
       <c r="B38" s="17" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C38" s="17" t="n">
         <v>7</v>
       </c>
       <c r="D38" s="18" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
@@ -1831,10 +1831,10 @@
         <v>150</v>
       </c>
       <c r="H38" s="19" t="n">
-        <v>47.33333333333334</v>
+        <v>48</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39">
@@ -1939,17 +1939,17 @@
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>Addada B.O</t>
+          <t>Lakshminarasimhapuram B.O</t>
         </is>
       </c>
       <c r="B42" s="17" t="n">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="C42" s="17" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="D42" s="18" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
@@ -1963,26 +1963,26 @@
         <v>150</v>
       </c>
       <c r="H42" s="19" t="n">
-        <v>42</v>
+        <v>43.33333333333334</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>Lakshminarasimhapuram B.O</t>
+          <t>Nuzella B.O</t>
         </is>
       </c>
       <c r="B43" s="17" t="n">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="C43" s="17" t="n">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="D43" s="18" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
@@ -1996,23 +1996,23 @@
         <v>150</v>
       </c>
       <c r="H43" s="19" t="n">
-        <v>42</v>
+        <v>42.66666666666667</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="16" t="inlineStr">
         <is>
-          <t>Nuzella B.O</t>
+          <t>Addada B.O</t>
         </is>
       </c>
       <c r="B44" s="17" t="n">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="C44" s="17" t="n">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="D44" s="18" t="n">
         <v>63</v>
@@ -2137,17 +2137,17 @@
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Chinayerukapadu B.O</t>
+          <t>Serigolvepalli B.O</t>
         </is>
       </c>
       <c r="B48" s="17" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="C48" s="17" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D48" s="18" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
@@ -2161,26 +2161,26 @@
         <v>150</v>
       </c>
       <c r="H48" s="19" t="n">
-        <v>38</v>
+        <v>38.66666666666666</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Lankapalli Agraharam B.O</t>
+          <t>Chinayerukapadu B.O</t>
         </is>
       </c>
       <c r="B49" s="17" t="n">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="C49" s="17" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
@@ -2194,26 +2194,26 @@
         <v>150</v>
       </c>
       <c r="H49" s="19" t="n">
-        <v>33.33333333333333</v>
+        <v>38</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>Polukonda B.O</t>
+          <t>Ramapuram B.O</t>
         </is>
       </c>
       <c r="B50" s="17" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="C50" s="17" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D50" s="18" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
@@ -2227,23 +2227,23 @@
         <v>150</v>
       </c>
       <c r="H50" s="19" t="n">
-        <v>33.33333333333333</v>
+        <v>34</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>Ramapuram B.O</t>
+          <t>Lankapalli Agraharam B.O</t>
         </is>
       </c>
       <c r="B51" s="17" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C51" s="17" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D51" s="18" t="n">
         <v>50</v>
@@ -2269,17 +2269,17 @@
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>Vanapumala B.O</t>
+          <t>Polukonda B.O</t>
         </is>
       </c>
       <c r="B52" s="17" t="n">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C52" s="17" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
@@ -2293,26 +2293,26 @@
         <v>150</v>
       </c>
       <c r="H52" s="19" t="n">
-        <v>32</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
         <is>
-          <t>Guraza B.O</t>
+          <t>Vanapumala B.O</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C53" s="17" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D53" s="18" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
@@ -2326,26 +2326,26 @@
         <v>150</v>
       </c>
       <c r="H53" s="19" t="n">
-        <v>31.33333333333334</v>
+        <v>32</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>Komarru B.O</t>
+          <t>Guraza B.O</t>
         </is>
       </c>
       <c r="B54" s="17" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="C54" s="17" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D54" s="18" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
@@ -2359,10 +2359,10 @@
         <v>150</v>
       </c>
       <c r="H54" s="19" t="n">
-        <v>30.66666666666666</v>
+        <v>31.33333333333334</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55">
@@ -2434,17 +2434,17 @@
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>Siddantham B.O</t>
+          <t>Komarru B.O</t>
         </is>
       </c>
       <c r="B57" s="17" t="n">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="C57" s="17" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="D57" s="18" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
@@ -2458,27 +2458,27 @@
         <v>150</v>
       </c>
       <c r="H57" s="19" t="n">
-        <v>26.66666666666667</v>
+        <v>29.33333333333333</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>Serigolvepalli B.O</t>
+          <t>Siddantham B.O</t>
         </is>
       </c>
       <c r="B58" s="17" t="n">
-        <v>78</v>
+        <v>133</v>
       </c>
       <c r="C58" s="17" t="n">
+        <v>93</v>
+      </c>
+      <c r="D58" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="D58" s="18" t="n">
-        <v>38</v>
-      </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
           <t>BO</t>
@@ -2491,10 +2491,10 @@
         <v>150</v>
       </c>
       <c r="H58" s="19" t="n">
-        <v>25.33333333333334</v>
+        <v>26.66666666666667</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59">
@@ -2867,13 +2867,13 @@
         </is>
       </c>
       <c r="B70" s="17" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C70" s="17" t="n">
         <v>14</v>
       </c>
       <c r="D70" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
@@ -2887,10 +2887,10 @@
         <v>150</v>
       </c>
       <c r="H70" s="19" t="n">
-        <v>2</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71">
@@ -2936,10 +2936,10 @@
         <v>250</v>
       </c>
       <c r="C72" s="17" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D72" s="18" t="n">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="E72" s="16" t="inlineStr">
         <is>
@@ -2953,10 +2953,10 @@
         <v>150</v>
       </c>
       <c r="H72" s="19" t="n">
-        <v>-5.333333333333334</v>
+        <v>-6</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73">
@@ -2999,13 +2999,13 @@
         </is>
       </c>
       <c r="B74" s="17" t="n">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="C74" s="17" t="n">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="D74" s="18" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E74" s="16" t="inlineStr">
         <is>
@@ -3019,10 +3019,10 @@
         <v>1000</v>
       </c>
       <c r="H74" s="19" t="n">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="75">
@@ -3035,10 +3035,10 @@
         <v>440</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
@@ -3052,7 +3052,7 @@
         <v>300</v>
       </c>
       <c r="H75" s="5" t="n">
-        <v>125.3333333333333</v>
+        <v>125</v>
       </c>
       <c r="I75" s="6" t="n">
         <v>0</v>
@@ -3131,13 +3131,13 @@
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="C78" s="8" t="n">
         <v>34</v>
       </c>
       <c r="D78" s="9" t="n">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -3151,10 +3151,10 @@
         <v>300</v>
       </c>
       <c r="H78" s="10" t="n">
-        <v>92.66666666666666</v>
+        <v>96</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79">
@@ -3230,10 +3230,10 @@
         </is>
       </c>
       <c r="B81" s="13" t="n">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C81" s="13" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D81" s="14" t="n">
         <v>234</v>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B83" s="13" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C83" s="13" t="n">
         <v>52</v>
       </c>
       <c r="D83" s="14" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E83" s="12" t="inlineStr">
         <is>
@@ -3316,10 +3316,10 @@
         <v>300</v>
       </c>
       <c r="H83" s="15" t="n">
-        <v>55.00000000000001</v>
+        <v>55.33333333333334</v>
       </c>
       <c r="I83" s="11" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="84">
@@ -3362,13 +3362,13 @@
         </is>
       </c>
       <c r="B85" s="17" t="n">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C85" s="17" t="n">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D85" s="18" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
@@ -3382,10 +3382,10 @@
         <v>300</v>
       </c>
       <c r="H85" s="19" t="n">
-        <v>49</v>
+        <v>49.33333333333334</v>
       </c>
       <c r="I85" s="11" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="86">
@@ -3497,10 +3497,10 @@
         <v>135</v>
       </c>
       <c r="C89" s="17" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D89" s="18" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
@@ -3514,10 +3514,10 @@
         <v>300</v>
       </c>
       <c r="H89" s="19" t="n">
-        <v>25.33333333333334</v>
+        <v>25</v>
       </c>
       <c r="I89" s="11" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -3694,52 +3694,52 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Bhushanagulla B.O</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>164</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>146</v>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H5" s="10" t="n">
-        <v>97.33333333333334</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>4</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Bollapadu B.O</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Dosapadu B.O</t>
+          <t>Bhushanagulla B.O</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -3753,26 +3753,26 @@
         <v>150</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>92.66666666666666</v>
+        <v>97.33333333333334</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Koyyagurapadu B.O</t>
+          <t>Dosapadu B.O</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
@@ -3786,26 +3786,26 @@
         <v>150</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>91.33333333333333</v>
+        <v>92.66666666666666</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Vemanda B.O</t>
+          <t>Koyyagurapadu B.O</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -3819,26 +3819,26 @@
         <v>150</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>88.66666666666667</v>
+        <v>91.33333333333333</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Bokinala B.O</t>
+          <t>Vemanda B.O</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
@@ -3852,26 +3852,26 @@
         <v>150</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>85.33333333333334</v>
+        <v>88.66666666666667</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Bollapadu B.O</t>
+          <t>Bokinala B.O</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>150</v>
+        <v>192</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
@@ -3885,26 +3885,26 @@
         <v>150</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>83.33333333333334</v>
+        <v>85.33333333333334</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Unikili B.O</t>
+          <t>Tummalapalli B.O</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
@@ -3918,92 +3918,92 @@
         <v>150</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>82</v>
+        <v>85.33333333333334</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
+          <t>Unikili B.O</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>123</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
           <t>Komatigunta Lock B.O</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B13" s="8" t="n">
         <v>191</v>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>69</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>122</v>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>81.33333333333333</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Pedapalaparru B.O</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>137</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>118</v>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>150</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>78.66666666666666</v>
+      <c r="C13" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>121</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>80.66666666666666</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Guruvindagunta B.O</t>
+          <t>Pedapalaparru B.O</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
@@ -4017,26 +4017,26 @@
         <v>150</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>75.33333333333333</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Chowtapalli B.O</t>
+          <t>Moparru B.O</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>171</v>
+        <v>133</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
@@ -4050,26 +4050,26 @@
         <v>150</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Moparru B.O</t>
+          <t>Guruvindagunta B.O</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
@@ -4083,59 +4083,59 @@
         <v>150</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>72.66666666666667</v>
+        <v>75.33333333333333</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Valivarthipadu B.O</t>
+          <t>Lingavaram B.O</t>
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="C17" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>111</v>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <v>74</v>
+      </c>
+      <c r="I17" s="11" t="n">
         <v>39</v>
-      </c>
-      <c r="D17" s="14" t="n">
-        <v>108</v>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F17" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>150</v>
-      </c>
-      <c r="H17" s="15" t="n">
-        <v>72</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>42</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Kanukollu B.O</t>
+          <t>Chowtapalli B.O</t>
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="D18" s="14" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
@@ -4149,23 +4149,23 @@
         <v>150</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Tativarru B.O</t>
+          <t>Valivarthipadu B.O</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>108</v>
@@ -4191,17 +4191,17 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Gunnanapudi B.O</t>
+          <t>Tativarru B.O</t>
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D20" s="14" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
@@ -4215,26 +4215,26 @@
         <v>150</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>70.66666666666667</v>
+        <v>72</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Lingavaram B.O</t>
+          <t>Kanukollu B.O</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D21" s="14" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
@@ -4248,26 +4248,26 @@
         <v>150</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Velinuthala B.O</t>
+          <t>Gunnanapudi B.O</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D22" s="14" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
@@ -4281,26 +4281,26 @@
         <v>150</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>67.33333333333333</v>
+        <v>70.66666666666667</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Gandhi Asramam B.O</t>
+          <t>Velinuthala B.O</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>107</v>
+        <v>154</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="D23" s="14" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
@@ -4314,10 +4314,10 @@
         <v>150</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>65.33333333333333</v>
+        <v>67.33333333333333</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
@@ -4356,17 +4356,17 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Garapadu B.O</t>
+          <t>Gandhi Asramam B.O</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D25" s="14" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
@@ -4380,26 +4380,26 @@
         <v>150</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>64.66666666666666</v>
+        <v>65.33333333333333</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Putlacheruvu B.O</t>
+          <t>Garapadu B.O</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="D26" s="14" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
@@ -4413,26 +4413,26 @@
         <v>150</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>64</v>
+        <v>64.66666666666666</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>Nandigamalanka B.O</t>
+          <t>Putlacheruvu B.O</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>104</v>
+        <v>137</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
@@ -4446,26 +4446,26 @@
         <v>150</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Ingilipakalanka B.O</t>
+          <t>Nandigamalanka B.O</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
@@ -4479,10 +4479,10 @@
         <v>150</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>59.33333333333334</v>
+        <v>62</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29">
@@ -4521,17 +4521,17 @@
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Bommuluru B.O</t>
+          <t>Ingilipakalanka B.O</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>156</v>
+        <v>112</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
@@ -4545,26 +4545,26 @@
         <v>150</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>58.66666666666666</v>
+        <v>59.33333333333334</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Tummalapalli B.O</t>
+          <t>Bommuluru B.O</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>128</v>
+        <v>156</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
@@ -4578,10 +4578,10 @@
         <v>150</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>56.00000000000001</v>
+        <v>58.66666666666666</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32">
@@ -4591,13 +4591,13 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>16</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
@@ -4611,10 +4611,10 @@
         <v>150</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>55.33333333333334</v>
+        <v>57.33333333333334</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33">
@@ -4789,13 +4789,13 @@
         </is>
       </c>
       <c r="B38" s="17" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C38" s="17" t="n">
         <v>7</v>
       </c>
       <c r="D38" s="18" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
@@ -4809,10 +4809,10 @@
         <v>150</v>
       </c>
       <c r="H38" s="19" t="n">
-        <v>47.33333333333334</v>
+        <v>48</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39">
@@ -4917,17 +4917,17 @@
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>Nuzella B.O</t>
+          <t>Lakshminarasimhapuram B.O</t>
         </is>
       </c>
       <c r="B42" s="17" t="n">
-        <v>122</v>
+        <v>74</v>
       </c>
       <c r="C42" s="17" t="n">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="D42" s="18" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
@@ -4941,26 +4941,26 @@
         <v>150</v>
       </c>
       <c r="H42" s="19" t="n">
-        <v>42</v>
+        <v>43.33333333333334</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>Lakshminarasimhapuram B.O</t>
+          <t>Nuzella B.O</t>
         </is>
       </c>
       <c r="B43" s="17" t="n">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="C43" s="17" t="n">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="D43" s="18" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
@@ -4974,10 +4974,10 @@
         <v>150</v>
       </c>
       <c r="H43" s="19" t="n">
-        <v>42</v>
+        <v>42.66666666666667</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44">
@@ -5115,17 +5115,17 @@
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Chinayerukapadu B.O</t>
+          <t>Serigolvepalli B.O</t>
         </is>
       </c>
       <c r="B48" s="17" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="C48" s="17" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D48" s="18" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
@@ -5139,26 +5139,26 @@
         <v>150</v>
       </c>
       <c r="H48" s="19" t="n">
-        <v>38</v>
+        <v>38.66666666666666</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Lankapalli Agraharam B.O</t>
+          <t>Chinayerukapadu B.O</t>
         </is>
       </c>
       <c r="B49" s="17" t="n">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="C49" s="17" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
@@ -5172,26 +5172,26 @@
         <v>150</v>
       </c>
       <c r="H49" s="19" t="n">
-        <v>33.33333333333333</v>
+        <v>38</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>Polukonda B.O</t>
+          <t>Ramapuram B.O</t>
         </is>
       </c>
       <c r="B50" s="17" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="C50" s="17" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D50" s="18" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
@@ -5205,23 +5205,23 @@
         <v>150</v>
       </c>
       <c r="H50" s="19" t="n">
-        <v>33.33333333333333</v>
+        <v>34</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>Ramapuram B.O</t>
+          <t>Lankapalli Agraharam B.O</t>
         </is>
       </c>
       <c r="B51" s="17" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C51" s="17" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D51" s="18" t="n">
         <v>50</v>
@@ -5247,17 +5247,17 @@
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>Vanapumala B.O</t>
+          <t>Polukonda B.O</t>
         </is>
       </c>
       <c r="B52" s="17" t="n">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C52" s="17" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
@@ -5271,26 +5271,26 @@
         <v>150</v>
       </c>
       <c r="H52" s="19" t="n">
-        <v>32</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
         <is>
-          <t>Guraza B.O</t>
+          <t>Vanapumala B.O</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C53" s="17" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D53" s="18" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
@@ -5304,26 +5304,26 @@
         <v>150</v>
       </c>
       <c r="H53" s="19" t="n">
-        <v>31.33333333333334</v>
+        <v>32</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>Komarru B.O</t>
+          <t>Guraza B.O</t>
         </is>
       </c>
       <c r="B54" s="17" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="C54" s="17" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D54" s="18" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
@@ -5337,10 +5337,10 @@
         <v>150</v>
       </c>
       <c r="H54" s="19" t="n">
-        <v>30.66666666666666</v>
+        <v>31.33333333333334</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55">
@@ -5379,14 +5379,14 @@
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>Chinapalaparru B.O</t>
+          <t>Komarru B.O</t>
         </is>
       </c>
       <c r="B56" s="17" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C56" s="17" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D56" s="18" t="n">
         <v>44</v>
@@ -5412,17 +5412,17 @@
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>Siddantham B.O</t>
+          <t>Chinapalaparru B.O</t>
         </is>
       </c>
       <c r="B57" s="17" t="n">
-        <v>133</v>
+        <v>74</v>
       </c>
       <c r="C57" s="17" t="n">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="D57" s="18" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
@@ -5436,27 +5436,27 @@
         <v>150</v>
       </c>
       <c r="H57" s="19" t="n">
-        <v>26.66666666666667</v>
+        <v>29.33333333333333</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>Serigolvepalli B.O</t>
+          <t>Siddantham B.O</t>
         </is>
       </c>
       <c r="B58" s="17" t="n">
-        <v>78</v>
+        <v>133</v>
       </c>
       <c r="C58" s="17" t="n">
+        <v>93</v>
+      </c>
+      <c r="D58" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="D58" s="18" t="n">
-        <v>38</v>
-      </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
           <t>BO</t>
@@ -5469,10 +5469,10 @@
         <v>150</v>
       </c>
       <c r="H58" s="19" t="n">
-        <v>25.33333333333334</v>
+        <v>26.66666666666667</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59">
@@ -5845,13 +5845,13 @@
         </is>
       </c>
       <c r="B70" s="17" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C70" s="17" t="n">
         <v>14</v>
       </c>
       <c r="D70" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
@@ -5865,10 +5865,10 @@
         <v>150</v>
       </c>
       <c r="H70" s="19" t="n">
-        <v>2</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71">
@@ -5914,10 +5914,10 @@
         <v>250</v>
       </c>
       <c r="C72" s="17" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D72" s="18" t="n">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="E72" s="16" t="inlineStr">
         <is>
@@ -5931,10 +5931,10 @@
         <v>150</v>
       </c>
       <c r="H72" s="19" t="n">
-        <v>-5.333333333333334</v>
+        <v>-6</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73">
@@ -6054,10 +6054,10 @@
         <v>440</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         <v>300</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>125.3333333333333</v>
+        <v>125</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -6150,13 +6150,13 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>34</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>300</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>92.66666666666666</v>
+        <v>96</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -6249,10 +6249,10 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D8" s="14" t="n">
         <v>234</v>
@@ -6315,13 +6315,13 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>52</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
@@ -6335,10 +6335,10 @@
         <v>300</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>55.00000000000001</v>
+        <v>55.33333333333334</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11">
@@ -6381,13 +6381,13 @@
         </is>
       </c>
       <c r="B12" s="17" t="n">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
@@ -6401,10 +6401,10 @@
         <v>300</v>
       </c>
       <c r="H12" s="19" t="n">
-        <v>49</v>
+        <v>49.33333333333334</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13">
@@ -6516,10 +6516,10 @@
         <v>135</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E16" s="16" t="inlineStr">
         <is>
@@ -6533,10 +6533,10 @@
         <v>300</v>
       </c>
       <c r="H16" s="19" t="n">
-        <v>25.33333333333334</v>
+        <v>25</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -6620,13 +6620,13 @@
         </is>
       </c>
       <c r="B2" s="17" t="n">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="D2" s="18" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
@@ -6640,10 +6640,10 @@
         <v>1000</v>
       </c>
       <c r="H2" s="19" t="n">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>
@@ -6822,17 +6822,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bhushanagulla B.O</t>
+          <t>Bollapadu B.O</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -6846,26 +6846,26 @@
         <v>150</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>97.33333333333334</v>
+        <v>100</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dosapadu B.O</t>
+          <t>Bhushanagulla B.O</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -6879,10 +6879,10 @@
         <v>150</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>92.66666666666666</v>
+        <v>97.33333333333334</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -7002,10 +7002,10 @@
         <v>250</v>
       </c>
       <c r="C3" s="17" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D3" s="18" t="n">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
@@ -7019,10 +7019,10 @@
         <v>150</v>
       </c>
       <c r="H3" s="19" t="n">
-        <v>-5.333333333333334</v>
+        <v>-6</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
@@ -7065,13 +7065,13 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>14</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
@@ -7085,10 +7085,10 @@
         <v>150</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>2</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6">
@@ -7208,10 +7208,10 @@
         <v>440</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -7225,7 +7225,7 @@
         <v>300</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>125.3333333333333</v>
+        <v>125</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -7381,10 +7381,10 @@
         <v>135</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D2" s="18" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
@@ -7398,10 +7398,10 @@
         <v>300</v>
       </c>
       <c r="H2" s="19" t="n">
-        <v>25.33333333333334</v>
+        <v>25</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -7568,7 +7568,7 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>14274</v>
+        <v>14404</v>
       </c>
     </row>
     <row r="8">
@@ -7578,7 +7578,7 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>5248</v>
+        <v>5261</v>
       </c>
     </row>
     <row r="9">
@@ -7588,7 +7588,7 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>9026</v>
+        <v>9143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update latest POSB data, Top of Mind and colour reports
</commit_message>
<xml_diff>
--- a/Gudivada_Net_Accounts_Latest.xlsx
+++ b/Gudivada_Net_Accounts_Latest.xlsx
@@ -659,10 +659,10 @@
         <v>239</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
         <v>150</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>130</v>
+        <v>123.3333333333333</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0</v>
@@ -692,10 +692,10 @@
         <v>253</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         <v>150</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>128.6666666666667</v>
+        <v>115.3333333333333</v>
       </c>
       <c r="I4" s="6" t="n">
         <v>0</v>
@@ -949,17 +949,17 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Vemanda B.O</t>
+          <t>Unikili B.O</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>180</v>
+        <v>161</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
@@ -973,26 +973,26 @@
         <v>150</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>91.33333333333333</v>
+        <v>94.66666666666667</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Pedapalaparru B.O</t>
+          <t>Nandamuru B.O</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>153</v>
+        <v>238</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>19</v>
+        <v>102</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
@@ -1006,59 +1006,59 @@
         <v>150</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>89.33333333333333</v>
+        <v>90.66666666666666</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Guruvindagunta B.O</t>
+          <t>Vemanda B.O</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="C14" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>136</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>90.66666666666666</v>
+      </c>
+      <c r="I14" s="11" t="n">
         <v>14</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>132</v>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>88</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Nandamuru B.O</t>
+          <t>Pedapalaparru B.O</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>228</v>
+        <v>153</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -1072,26 +1072,26 @@
         <v>150</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>85.33333333333334</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Kanukollu B.O</t>
+          <t>Guruvindagunta B.O</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -1105,26 +1105,26 @@
         <v>150</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Lingavaram B.O</t>
+          <t>Kanukollu B.O</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -1138,26 +1138,26 @@
         <v>150</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>82.66666666666667</v>
+        <v>84</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Komatigunta Lock B.O</t>
+          <t>Lingavaram B.O</t>
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>194</v>
+        <v>144</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
@@ -1171,26 +1171,26 @@
         <v>150</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>82</v>
+        <v>82.66666666666667</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Unikili B.O</t>
+          <t>Putlacheruvu B.O</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
@@ -1204,43 +1204,43 @@
         <v>150</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>81.33333333333333</v>
+        <v>80.66666666666666</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Tativarru B.O</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="n">
-        <v>148</v>
-      </c>
-      <c r="C20" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>119</v>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G20" s="13" t="n">
-        <v>150</v>
-      </c>
-      <c r="H20" s="15" t="n">
-        <v>79.33333333333333</v>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Komatigunta Lock B.O</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>194</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>80</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
@@ -1312,17 +1312,17 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Chowtapalli B.O</t>
+          <t>Tativarru B.O</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>171</v>
+        <v>148</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="D23" s="14" t="n">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
@@ -1336,26 +1336,26 @@
         <v>150</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>72</v>
+        <v>76.66666666666667</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Bommuluru B.O</t>
+          <t>Chowtapalli B.O</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D24" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
@@ -1369,10 +1369,10 @@
         <v>150</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>71.33333333333334</v>
+        <v>72</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25">
@@ -1411,17 +1411,17 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Tenneru B.O</t>
+          <t>Gandhi Asramam B.O</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>273</v>
+        <v>112</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="D26" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
@@ -1435,26 +1435,26 @@
         <v>150</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>68</v>
+        <v>68.66666666666667</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>Vadali B.O</t>
+          <t>Velinuthala B.O</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
@@ -1468,26 +1468,26 @@
         <v>150</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>68</v>
+        <v>68.66666666666667</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Gandhi Asramam B.O</t>
+          <t>Tenneru B.O</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>107</v>
+        <v>273</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>9</v>
+        <v>171</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
@@ -1501,26 +1501,26 @@
         <v>150</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>65.33333333333333</v>
+        <v>68</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>Putlacheruvu B.O</t>
+          <t>Vadali B.O</t>
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
@@ -1534,26 +1534,26 @@
         <v>150</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Velinuthala B.O</t>
+          <t>Komaravolu B.O</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
@@ -1567,26 +1567,26 @@
         <v>150</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>64</v>
+        <v>63.33333333333333</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Komaravolu B.O</t>
+          <t>Polukonda B.O</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>180</v>
+        <v>126</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
@@ -1600,26 +1600,26 @@
         <v>150</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>63.33333333333333</v>
+        <v>58.66666666666666</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Garapadu B.O</t>
+          <t>Bommuluru B.O</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>113</v>
+        <v>178</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
@@ -1633,26 +1633,26 @@
         <v>150</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>58.66666666666666</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Polukonda B.O</t>
+          <t>Veldipadu B.O</t>
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="C33" s="13" t="n">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="D33" s="14" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
@@ -1666,26 +1666,26 @@
         <v>150</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>58.66666666666666</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Veldipadu B.O</t>
+          <t>Lankapalli Agraharam B.O</t>
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="D34" s="14" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
@@ -1699,10 +1699,10 @@
         <v>150</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>57.99999999999999</v>
+        <v>57.33333333333334</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35">
@@ -1814,10 +1814,10 @@
         <v>117</v>
       </c>
       <c r="C38" s="13" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D38" s="14" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
@@ -1831,23 +1831,23 @@
         <v>150</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>55.33333333333334</v>
+        <v>54</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Lankapalli Agraharam B.O</t>
+          <t>Nandivada B.O</t>
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C39" s="13" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D39" s="14" t="n">
         <v>80</v>
@@ -1873,14 +1873,14 @@
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>Nandivada B.O</t>
+          <t>Ramapuram B.O</t>
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>80</v>
@@ -1976,13 +1976,13 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C43" s="13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D43" s="14" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
@@ -1996,23 +1996,23 @@
         <v>150</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>50</v>
+        <v>50.66666666666667</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>Ponukumadu B.O</t>
+          <t>Chinayerukapadu B.O</t>
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C44" s="13" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="D44" s="14" t="n">
         <v>75</v>
@@ -2036,52 +2036,52 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>Pedakamanapudi B.O</t>
-        </is>
-      </c>
-      <c r="B45" s="17" t="n">
-        <v>104</v>
-      </c>
-      <c r="C45" s="17" t="n">
-        <v>31</v>
-      </c>
-      <c r="D45" s="18" t="n">
-        <v>73</v>
-      </c>
-      <c r="E45" s="16" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F45" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G45" s="17" t="n">
-        <v>150</v>
-      </c>
-      <c r="H45" s="19" t="n">
-        <v>48.66666666666667</v>
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Ponukumadu B.O</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="n">
+        <v>102</v>
+      </c>
+      <c r="C45" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F45" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G45" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="H45" s="15" t="n">
+        <v>50</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>Dondapadu B.O</t>
+          <t>Siddantham B.O</t>
         </is>
       </c>
       <c r="B46" s="17" t="n">
-        <v>119</v>
+        <v>168</v>
       </c>
       <c r="C46" s="17" t="n">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="D46" s="18" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
@@ -2095,26 +2095,26 @@
         <v>150</v>
       </c>
       <c r="H46" s="19" t="n">
-        <v>47.33333333333334</v>
+        <v>49.33333333333334</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>Guraza B.O</t>
+          <t>Addada B.O</t>
         </is>
       </c>
       <c r="B47" s="17" t="n">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="C47" s="17" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D47" s="18" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
@@ -2128,26 +2128,26 @@
         <v>150</v>
       </c>
       <c r="H47" s="19" t="n">
-        <v>47.33333333333334</v>
+        <v>48.66666666666667</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Edulamaddali B.O</t>
+          <t>Pedakamanapudi B.O</t>
         </is>
       </c>
       <c r="B48" s="17" t="n">
-        <v>149</v>
+        <v>104</v>
       </c>
       <c r="C48" s="17" t="n">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="D48" s="18" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
@@ -2161,26 +2161,26 @@
         <v>150</v>
       </c>
       <c r="H48" s="19" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Ramapuram B.O</t>
+          <t>Guraza B.O</t>
         </is>
       </c>
       <c r="B49" s="17" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C49" s="17" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
@@ -2194,26 +2194,26 @@
         <v>150</v>
       </c>
       <c r="H49" s="19" t="n">
-        <v>46</v>
+        <v>47.33333333333334</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>Chinapalaparru B.O</t>
+          <t>Dondapadu B.O</t>
         </is>
       </c>
       <c r="B50" s="17" t="n">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C50" s="17" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D50" s="18" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
@@ -2227,26 +2227,26 @@
         <v>150</v>
       </c>
       <c r="H50" s="19" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>Chinayerukapadu B.O</t>
+          <t>Lakshminarasimhapuram B.O</t>
         </is>
       </c>
       <c r="B51" s="17" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="C51" s="17" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D51" s="18" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
@@ -2260,23 +2260,23 @@
         <v>150</v>
       </c>
       <c r="H51" s="19" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>Lakshminarasimhapuram B.O</t>
+          <t>Chinapalaparru B.O</t>
         </is>
       </c>
       <c r="B52" s="17" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="C52" s="17" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="D52" s="18" t="n">
         <v>66</v>
@@ -2335,17 +2335,17 @@
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>Siddantham B.O</t>
+          <t>Sankarshanapuram B.O</t>
         </is>
       </c>
       <c r="B54" s="17" t="n">
-        <v>158</v>
+        <v>64</v>
       </c>
       <c r="C54" s="17" t="n">
-        <v>94</v>
+        <v>5</v>
       </c>
       <c r="D54" s="18" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
@@ -2359,26 +2359,26 @@
         <v>150</v>
       </c>
       <c r="H54" s="19" t="n">
-        <v>42.66666666666667</v>
+        <v>39.33333333333333</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>Addada B.O</t>
+          <t>Serikalavapudi B.O</t>
         </is>
       </c>
       <c r="B55" s="17" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="C55" s="17" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D55" s="18" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
@@ -2392,26 +2392,26 @@
         <v>150</v>
       </c>
       <c r="H55" s="19" t="n">
-        <v>42</v>
+        <v>39.33333333333333</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>Serikalavapudi B.O</t>
+          <t>Vempadu B.O</t>
         </is>
       </c>
       <c r="B56" s="17" t="n">
-        <v>87</v>
+        <v>155</v>
       </c>
       <c r="C56" s="17" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="D56" s="18" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
@@ -2425,26 +2425,26 @@
         <v>150</v>
       </c>
       <c r="H56" s="19" t="n">
-        <v>39.33333333333333</v>
+        <v>38.66666666666666</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>Serigolvepalli B.O</t>
+          <t>Amudalapalli B.O</t>
         </is>
       </c>
       <c r="B57" s="17" t="n">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="C57" s="17" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D57" s="18" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
@@ -2458,26 +2458,26 @@
         <v>150</v>
       </c>
       <c r="H57" s="19" t="n">
-        <v>38.66666666666666</v>
+        <v>38</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>Amudalapalli B.O</t>
+          <t>Peruru B.O</t>
         </is>
       </c>
       <c r="B58" s="17" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C58" s="17" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D58" s="18" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
@@ -2491,26 +2491,26 @@
         <v>150</v>
       </c>
       <c r="H58" s="19" t="n">
-        <v>38</v>
+        <v>36.66666666666666</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>Peruru B.O</t>
+          <t>Vanapumala B.O</t>
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C59" s="17" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="D59" s="18" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
@@ -2524,26 +2524,26 @@
         <v>150</v>
       </c>
       <c r="H59" s="19" t="n">
-        <v>37.33333333333334</v>
+        <v>36</v>
       </c>
       <c r="I59" s="11" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>Sankarshanapuram B.O</t>
+          <t>Edulamaddali B.O</t>
         </is>
       </c>
       <c r="B60" s="17" t="n">
-        <v>59</v>
+        <v>149</v>
       </c>
       <c r="C60" s="17" t="n">
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="D60" s="18" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
@@ -2557,26 +2557,26 @@
         <v>150</v>
       </c>
       <c r="H60" s="19" t="n">
-        <v>36</v>
+        <v>35.33333333333334</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>Vanapumala B.O</t>
+          <t>K.P.Agraharam B.O</t>
         </is>
       </c>
       <c r="B61" s="17" t="n">
-        <v>69</v>
+        <v>176</v>
       </c>
       <c r="C61" s="17" t="n">
-        <v>15</v>
+        <v>123</v>
       </c>
       <c r="D61" s="18" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
@@ -2590,26 +2590,26 @@
         <v>150</v>
       </c>
       <c r="H61" s="19" t="n">
-        <v>36</v>
+        <v>35.33333333333334</v>
       </c>
       <c r="I61" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
         <is>
-          <t>K.P.Agraharam B.O</t>
+          <t>Chandrala B.O</t>
         </is>
       </c>
       <c r="B62" s="17" t="n">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="C62" s="17" t="n">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="D62" s="18" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
@@ -2623,10 +2623,10 @@
         <v>150</v>
       </c>
       <c r="H62" s="19" t="n">
-        <v>35.33333333333334</v>
+        <v>34.66666666666667</v>
       </c>
       <c r="I62" s="11" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="63">
@@ -2665,17 +2665,17 @@
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
         <is>
-          <t>Komarru B.O</t>
+          <t>Garapadu B.O</t>
         </is>
       </c>
       <c r="B64" s="17" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C64" s="17" t="n">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D64" s="18" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E64" s="16" t="inlineStr">
         <is>
@@ -2689,26 +2689,26 @@
         <v>150</v>
       </c>
       <c r="H64" s="19" t="n">
-        <v>32.66666666666666</v>
+        <v>32</v>
       </c>
       <c r="I64" s="11" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>Billapadu</t>
+          <t>Komarru B.O</t>
         </is>
       </c>
       <c r="B65" s="17" t="n">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="C65" s="17" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="D65" s="18" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
@@ -2722,26 +2722,26 @@
         <v>150</v>
       </c>
       <c r="H65" s="19" t="n">
-        <v>22.66666666666666</v>
+        <v>32</v>
       </c>
       <c r="I65" s="11" t="n">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
         <is>
-          <t>Chandrala B.O</t>
+          <t>Serigolvepalli B.O</t>
         </is>
       </c>
       <c r="B66" s="17" t="n">
-        <v>170</v>
+        <v>98</v>
       </c>
       <c r="C66" s="17" t="n">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="D66" s="18" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
@@ -2755,26 +2755,26 @@
         <v>150</v>
       </c>
       <c r="H66" s="19" t="n">
-        <v>21.33333333333334</v>
+        <v>25.33333333333334</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
         <is>
-          <t>Lingala B.O</t>
+          <t>Billapadu</t>
         </is>
       </c>
       <c r="B67" s="17" t="n">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="C67" s="17" t="n">
-        <v>68</v>
+        <v>19</v>
       </c>
       <c r="D67" s="18" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
@@ -2788,10 +2788,10 @@
         <v>150</v>
       </c>
       <c r="H67" s="19" t="n">
-        <v>21.33333333333334</v>
+        <v>22.66666666666666</v>
       </c>
       <c r="I67" s="11" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="68">
@@ -2801,13 +2801,13 @@
         </is>
       </c>
       <c r="B68" s="17" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C68" s="17" t="n">
         <v>50</v>
       </c>
       <c r="D68" s="18" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
@@ -2821,26 +2821,26 @@
         <v>150</v>
       </c>
       <c r="H68" s="19" t="n">
-        <v>20.66666666666667</v>
+        <v>22</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>Vempadu B.O</t>
+          <t>Lingala B.O</t>
         </is>
       </c>
       <c r="B69" s="17" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C69" s="17" t="n">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="D69" s="18" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
@@ -2854,10 +2854,10 @@
         <v>150</v>
       </c>
       <c r="H69" s="19" t="n">
-        <v>18.66666666666667</v>
+        <v>21.33333333333334</v>
       </c>
       <c r="I69" s="11" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="70">
@@ -2969,10 +2969,10 @@
         <v>6</v>
       </c>
       <c r="C73" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D73" s="18" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
@@ -2986,10 +2986,10 @@
         <v>150</v>
       </c>
       <c r="H73" s="19" t="n">
-        <v>-3.333333333333333</v>
+        <v>-4.666666666666667</v>
       </c>
       <c r="I73" s="11" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="74">
@@ -2999,13 +2999,13 @@
         </is>
       </c>
       <c r="B74" s="13" t="n">
-        <v>1430</v>
+        <v>1457</v>
       </c>
       <c r="C74" s="13" t="n">
-        <v>918</v>
+        <v>947</v>
       </c>
       <c r="D74" s="14" t="n">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
@@ -3019,10 +3019,10 @@
         <v>1000</v>
       </c>
       <c r="H74" s="15" t="n">
-        <v>51.2</v>
+        <v>51</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="75">
@@ -3032,13 +3032,13 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
@@ -3052,7 +3052,7 @@
         <v>300</v>
       </c>
       <c r="H75" s="5" t="n">
-        <v>125.6666666666667</v>
+        <v>125.3333333333333</v>
       </c>
       <c r="I75" s="6" t="n">
         <v>0</v>
@@ -3065,13 +3065,13 @@
         </is>
       </c>
       <c r="B76" s="3" t="n">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C76" s="3" t="n">
         <v>56</v>
       </c>
       <c r="D76" s="4" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
@@ -3085,7 +3085,7 @@
         <v>300</v>
       </c>
       <c r="H76" s="5" t="n">
-        <v>117.3333333333333</v>
+        <v>117.6666666666667</v>
       </c>
       <c r="I76" s="6" t="n">
         <v>0</v>
@@ -3098,13 +3098,13 @@
         </is>
       </c>
       <c r="B77" s="3" t="n">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C77" s="3" t="n">
         <v>68</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
@@ -3118,7 +3118,7 @@
         <v>300</v>
       </c>
       <c r="H77" s="5" t="n">
-        <v>105.3333333333333</v>
+        <v>106</v>
       </c>
       <c r="I77" s="6" t="n">
         <v>0</v>
@@ -3127,17 +3127,17 @@
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>Moturu S.O</t>
+          <t>Rudrapaka S.O</t>
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>355</v>
+        <v>328</v>
       </c>
       <c r="C78" s="8" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D78" s="9" t="n">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -3151,26 +3151,26 @@
         <v>300</v>
       </c>
       <c r="H78" s="10" t="n">
-        <v>99.33333333333333</v>
+        <v>97.66666666666667</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>Rudrapaka S.O</t>
+          <t>Moturu S.O</t>
         </is>
       </c>
       <c r="B79" s="8" t="n">
-        <v>328</v>
+        <v>356</v>
       </c>
       <c r="C79" s="8" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="D79" s="9" t="n">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
@@ -3184,10 +3184,10 @@
         <v>300</v>
       </c>
       <c r="H79" s="10" t="n">
-        <v>97.66666666666667</v>
+        <v>97.33333333333334</v>
       </c>
       <c r="I79" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
@@ -3197,13 +3197,13 @@
         </is>
       </c>
       <c r="B80" s="8" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C80" s="8" t="n">
         <v>96</v>
       </c>
       <c r="D80" s="9" t="n">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -3217,10 +3217,10 @@
         <v>300</v>
       </c>
       <c r="H80" s="10" t="n">
-        <v>90.33333333333333</v>
+        <v>92.33333333333333</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="81">
@@ -3230,13 +3230,13 @@
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>538</v>
+        <v>561</v>
       </c>
       <c r="C81" s="8" t="n">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="D81" s="9" t="n">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
@@ -3250,10 +3250,10 @@
         <v>300</v>
       </c>
       <c r="H81" s="10" t="n">
-        <v>83.66666666666667</v>
+        <v>88</v>
       </c>
       <c r="I81" s="11" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="82">
@@ -3263,13 +3263,13 @@
         </is>
       </c>
       <c r="B82" s="13" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C82" s="13" t="n">
         <v>31</v>
       </c>
       <c r="D82" s="14" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
@@ -3283,10 +3283,10 @@
         <v>300</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>71.66666666666667</v>
+        <v>72</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="83">
@@ -3362,13 +3362,13 @@
         </is>
       </c>
       <c r="B85" s="13" t="n">
-        <v>396</v>
+        <v>405</v>
       </c>
       <c r="C85" s="13" t="n">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D85" s="14" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E85" s="12" t="inlineStr">
         <is>
@@ -3382,10 +3382,10 @@
         <v>300</v>
       </c>
       <c r="H85" s="15" t="n">
-        <v>53.33333333333334</v>
+        <v>55.33333333333334</v>
       </c>
       <c r="I85" s="11" t="n">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="86">
@@ -3395,13 +3395,13 @@
         </is>
       </c>
       <c r="B86" s="17" t="n">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C86" s="17" t="n">
         <v>14</v>
       </c>
       <c r="D86" s="18" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E86" s="16" t="inlineStr">
         <is>
@@ -3415,10 +3415,10 @@
         <v>300</v>
       </c>
       <c r="H86" s="19" t="n">
-        <v>46</v>
+        <v>47.66666666666667</v>
       </c>
       <c r="I86" s="11" t="n">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="87">
@@ -3428,13 +3428,13 @@
         </is>
       </c>
       <c r="B87" s="17" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C87" s="17" t="n">
         <v>62</v>
       </c>
       <c r="D87" s="18" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
@@ -3448,10 +3448,10 @@
         <v>300</v>
       </c>
       <c r="H87" s="19" t="n">
-        <v>38.66666666666666</v>
+        <v>39</v>
       </c>
       <c r="I87" s="11" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="88">
@@ -3637,10 +3637,10 @@
         <v>239</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -3654,7 +3654,7 @@
         <v>150</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>130</v>
+        <v>123.3333333333333</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0</v>
@@ -3670,10 +3670,10 @@
         <v>253</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>150</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>128.6666666666667</v>
+        <v>115.3333333333333</v>
       </c>
       <c r="I4" s="6" t="n">
         <v>0</v>
@@ -3927,17 +3927,17 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Vemanda B.O</t>
+          <t>Unikili B.O</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>180</v>
+        <v>161</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
@@ -3951,26 +3951,26 @@
         <v>150</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>91.33333333333333</v>
+        <v>94.66666666666667</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Pedapalaparru B.O</t>
+          <t>Nandamuru B.O</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>153</v>
+        <v>238</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>19</v>
+        <v>102</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
@@ -3984,59 +3984,59 @@
         <v>150</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>89.33333333333333</v>
+        <v>90.66666666666666</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Guruvindagunta B.O</t>
+          <t>Vemanda B.O</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="C14" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>136</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>90.66666666666666</v>
+      </c>
+      <c r="I14" s="11" t="n">
         <v>14</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>132</v>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="n">
-        <v>300</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>88</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Nandamuru B.O</t>
+          <t>Pedapalaparru B.O</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>228</v>
+        <v>153</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -4050,26 +4050,26 @@
         <v>150</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>85.33333333333334</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Kanukollu B.O</t>
+          <t>Guruvindagunta B.O</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -4083,26 +4083,26 @@
         <v>150</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Lingavaram B.O</t>
+          <t>Kanukollu B.O</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -4116,26 +4116,26 @@
         <v>150</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>82.66666666666667</v>
+        <v>84</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Komatigunta Lock B.O</t>
+          <t>Lingavaram B.O</t>
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>194</v>
+        <v>144</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
@@ -4149,26 +4149,26 @@
         <v>150</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>82</v>
+        <v>82.66666666666667</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Unikili B.O</t>
+          <t>Putlacheruvu B.O</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
@@ -4182,43 +4182,43 @@
         <v>150</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>81.33333333333333</v>
+        <v>80.66666666666666</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Tativarru B.O</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="n">
-        <v>148</v>
-      </c>
-      <c r="C20" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>119</v>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G20" s="13" t="n">
-        <v>150</v>
-      </c>
-      <c r="H20" s="15" t="n">
-        <v>79.33333333333333</v>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Komatigunta Lock B.O</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>194</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>80</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
@@ -4290,17 +4290,17 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Chowtapalli B.O</t>
+          <t>Tativarru B.O</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>171</v>
+        <v>148</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="D23" s="14" t="n">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
@@ -4314,26 +4314,26 @@
         <v>150</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>72</v>
+        <v>76.66666666666667</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Bommuluru B.O</t>
+          <t>Chowtapalli B.O</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D24" s="14" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
@@ -4347,10 +4347,10 @@
         <v>150</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>71.33333333333334</v>
+        <v>72</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25">
@@ -4389,17 +4389,17 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Tenneru B.O</t>
+          <t>Gandhi Asramam B.O</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>273</v>
+        <v>112</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="D26" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
@@ -4413,26 +4413,26 @@
         <v>150</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>68</v>
+        <v>68.66666666666667</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>Vadali B.O</t>
+          <t>Velinuthala B.O</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
@@ -4446,26 +4446,26 @@
         <v>150</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>68</v>
+        <v>68.66666666666667</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Gandhi Asramam B.O</t>
+          <t>Tenneru B.O</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>107</v>
+        <v>273</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>9</v>
+        <v>171</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
@@ -4479,26 +4479,26 @@
         <v>150</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>65.33333333333333</v>
+        <v>68</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>Putlacheruvu B.O</t>
+          <t>Vadali B.O</t>
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
@@ -4512,26 +4512,26 @@
         <v>150</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Velinuthala B.O</t>
+          <t>Komaravolu B.O</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
@@ -4545,26 +4545,26 @@
         <v>150</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>64</v>
+        <v>63.33333333333333</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Komaravolu B.O</t>
+          <t>Polukonda B.O</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>180</v>
+        <v>126</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
@@ -4578,26 +4578,26 @@
         <v>150</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>63.33333333333333</v>
+        <v>58.66666666666666</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Polukonda B.O</t>
+          <t>Bommuluru B.O</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>126</v>
+        <v>178</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
@@ -4611,26 +4611,26 @@
         <v>150</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>58.66666666666666</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Garapadu B.O</t>
+          <t>Veldipadu B.O</t>
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="C33" s="13" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="D33" s="14" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
@@ -4644,26 +4644,26 @@
         <v>150</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>58.66666666666666</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Veldipadu B.O</t>
+          <t>Lankapalli Agraharam B.O</t>
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="D34" s="14" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
@@ -4677,10 +4677,10 @@
         <v>150</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>57.99999999999999</v>
+        <v>57.33333333333334</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35">
@@ -4792,10 +4792,10 @@
         <v>117</v>
       </c>
       <c r="C38" s="13" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D38" s="14" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
@@ -4809,23 +4809,23 @@
         <v>150</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>55.33333333333334</v>
+        <v>54</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Nandivada B.O</t>
+          <t>Ramapuram B.O</t>
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C39" s="13" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D39" s="14" t="n">
         <v>80</v>
@@ -4851,14 +4851,14 @@
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>Lankapalli Agraharam B.O</t>
+          <t>Nandivada B.O</t>
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>80</v>
@@ -4917,14 +4917,14 @@
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t>Nuzella B.O</t>
+          <t>Pedavirivada B.O</t>
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>138</v>
+        <v>84</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="D42" s="14" t="n">
         <v>76</v>
@@ -4950,17 +4950,17 @@
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>Pedavirivada B.O</t>
+          <t>Nuzella B.O</t>
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="C43" s="13" t="n">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="D43" s="14" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
@@ -4974,10 +4974,10 @@
         <v>150</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>50</v>
+        <v>50.66666666666667</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44">
@@ -5014,52 +5014,52 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>Pedakamanapudi B.O</t>
-        </is>
-      </c>
-      <c r="B45" s="17" t="n">
-        <v>104</v>
-      </c>
-      <c r="C45" s="17" t="n">
-        <v>31</v>
-      </c>
-      <c r="D45" s="18" t="n">
-        <v>73</v>
-      </c>
-      <c r="E45" s="16" t="inlineStr">
-        <is>
-          <t>BO</t>
-        </is>
-      </c>
-      <c r="F45" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G45" s="17" t="n">
-        <v>150</v>
-      </c>
-      <c r="H45" s="19" t="n">
-        <v>48.66666666666667</v>
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Chinayerukapadu B.O</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="n">
+        <v>110</v>
+      </c>
+      <c r="C45" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="F45" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G45" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="H45" s="15" t="n">
+        <v>50</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>Dondapadu B.O</t>
+          <t>Siddantham B.O</t>
         </is>
       </c>
       <c r="B46" s="17" t="n">
-        <v>119</v>
+        <v>168</v>
       </c>
       <c r="C46" s="17" t="n">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="D46" s="18" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
@@ -5073,26 +5073,26 @@
         <v>150</v>
       </c>
       <c r="H46" s="19" t="n">
-        <v>47.33333333333334</v>
+        <v>49.33333333333334</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>Guraza B.O</t>
+          <t>Addada B.O</t>
         </is>
       </c>
       <c r="B47" s="17" t="n">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="C47" s="17" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D47" s="18" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
@@ -5106,26 +5106,26 @@
         <v>150</v>
       </c>
       <c r="H47" s="19" t="n">
-        <v>47.33333333333334</v>
+        <v>48.66666666666667</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>Edulamaddali B.O</t>
+          <t>Pedakamanapudi B.O</t>
         </is>
       </c>
       <c r="B48" s="17" t="n">
-        <v>149</v>
+        <v>104</v>
       </c>
       <c r="C48" s="17" t="n">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="D48" s="18" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
@@ -5139,26 +5139,26 @@
         <v>150</v>
       </c>
       <c r="H48" s="19" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Ramapuram B.O</t>
+          <t>Guraza B.O</t>
         </is>
       </c>
       <c r="B49" s="17" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C49" s="17" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
@@ -5172,26 +5172,26 @@
         <v>150</v>
       </c>
       <c r="H49" s="19" t="n">
-        <v>46</v>
+        <v>47.33333333333334</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>Chinapalaparru B.O</t>
+          <t>Dondapadu B.O</t>
         </is>
       </c>
       <c r="B50" s="17" t="n">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="C50" s="17" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D50" s="18" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
@@ -5205,26 +5205,26 @@
         <v>150</v>
       </c>
       <c r="H50" s="19" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>Chinayerukapadu B.O</t>
+          <t>Lakshminarasimhapuram B.O</t>
         </is>
       </c>
       <c r="B51" s="17" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="C51" s="17" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D51" s="18" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
@@ -5238,23 +5238,23 @@
         <v>150</v>
       </c>
       <c r="H51" s="19" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>Lakshminarasimhapuram B.O</t>
+          <t>Chinapalaparru B.O</t>
         </is>
       </c>
       <c r="B52" s="17" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="C52" s="17" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="D52" s="18" t="n">
         <v>66</v>
@@ -5313,17 +5313,17 @@
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>Siddantham B.O</t>
+          <t>Sankarshanapuram B.O</t>
         </is>
       </c>
       <c r="B54" s="17" t="n">
-        <v>158</v>
+        <v>64</v>
       </c>
       <c r="C54" s="17" t="n">
-        <v>94</v>
+        <v>5</v>
       </c>
       <c r="D54" s="18" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
@@ -5337,26 +5337,26 @@
         <v>150</v>
       </c>
       <c r="H54" s="19" t="n">
-        <v>42.66666666666667</v>
+        <v>39.33333333333333</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>Addada B.O</t>
+          <t>Serikalavapudi B.O</t>
         </is>
       </c>
       <c r="B55" s="17" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="C55" s="17" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D55" s="18" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
@@ -5370,26 +5370,26 @@
         <v>150</v>
       </c>
       <c r="H55" s="19" t="n">
-        <v>42</v>
+        <v>39.33333333333333</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>Serikalavapudi B.O</t>
+          <t>Vempadu B.O</t>
         </is>
       </c>
       <c r="B56" s="17" t="n">
-        <v>87</v>
+        <v>155</v>
       </c>
       <c r="C56" s="17" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="D56" s="18" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
@@ -5403,26 +5403,26 @@
         <v>150</v>
       </c>
       <c r="H56" s="19" t="n">
-        <v>39.33333333333333</v>
+        <v>38.66666666666666</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>Serigolvepalli B.O</t>
+          <t>Amudalapalli B.O</t>
         </is>
       </c>
       <c r="B57" s="17" t="n">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="C57" s="17" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D57" s="18" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
@@ -5436,26 +5436,26 @@
         <v>150</v>
       </c>
       <c r="H57" s="19" t="n">
-        <v>38.66666666666666</v>
+        <v>38</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>Amudalapalli B.O</t>
+          <t>Peruru B.O</t>
         </is>
       </c>
       <c r="B58" s="17" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C58" s="17" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D58" s="18" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
@@ -5469,26 +5469,26 @@
         <v>150</v>
       </c>
       <c r="H58" s="19" t="n">
-        <v>38</v>
+        <v>36.66666666666666</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>Peruru B.O</t>
+          <t>Vanapumala B.O</t>
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C59" s="17" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="D59" s="18" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
@@ -5502,26 +5502,26 @@
         <v>150</v>
       </c>
       <c r="H59" s="19" t="n">
-        <v>37.33333333333334</v>
+        <v>36</v>
       </c>
       <c r="I59" s="11" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>Vanapumala B.O</t>
+          <t>Edulamaddali B.O</t>
         </is>
       </c>
       <c r="B60" s="17" t="n">
-        <v>69</v>
+        <v>149</v>
       </c>
       <c r="C60" s="17" t="n">
-        <v>15</v>
+        <v>96</v>
       </c>
       <c r="D60" s="18" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
@@ -5535,26 +5535,26 @@
         <v>150</v>
       </c>
       <c r="H60" s="19" t="n">
-        <v>36</v>
+        <v>35.33333333333334</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>Sankarshanapuram B.O</t>
+          <t>K.P.Agraharam B.O</t>
         </is>
       </c>
       <c r="B61" s="17" t="n">
-        <v>59</v>
+        <v>176</v>
       </c>
       <c r="C61" s="17" t="n">
-        <v>5</v>
+        <v>123</v>
       </c>
       <c r="D61" s="18" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
@@ -5568,26 +5568,26 @@
         <v>150</v>
       </c>
       <c r="H61" s="19" t="n">
-        <v>36</v>
+        <v>35.33333333333334</v>
       </c>
       <c r="I61" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
         <is>
-          <t>K.P.Agraharam B.O</t>
+          <t>Chandrala B.O</t>
         </is>
       </c>
       <c r="B62" s="17" t="n">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="C62" s="17" t="n">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="D62" s="18" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
@@ -5601,10 +5601,10 @@
         <v>150</v>
       </c>
       <c r="H62" s="19" t="n">
-        <v>35.33333333333334</v>
+        <v>34.66666666666667</v>
       </c>
       <c r="I62" s="11" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="63">
@@ -5643,17 +5643,17 @@
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
         <is>
-          <t>Komarru B.O</t>
+          <t>Garapadu B.O</t>
         </is>
       </c>
       <c r="B64" s="17" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C64" s="17" t="n">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D64" s="18" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E64" s="16" t="inlineStr">
         <is>
@@ -5667,26 +5667,26 @@
         <v>150</v>
       </c>
       <c r="H64" s="19" t="n">
-        <v>32.66666666666666</v>
+        <v>32</v>
       </c>
       <c r="I64" s="11" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>Billapadu</t>
+          <t>Komarru B.O</t>
         </is>
       </c>
       <c r="B65" s="17" t="n">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="C65" s="17" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="D65" s="18" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
@@ -5700,26 +5700,26 @@
         <v>150</v>
       </c>
       <c r="H65" s="19" t="n">
-        <v>22.66666666666666</v>
+        <v>32</v>
       </c>
       <c r="I65" s="11" t="n">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
         <is>
-          <t>Lingala B.O</t>
+          <t>Serigolvepalli B.O</t>
         </is>
       </c>
       <c r="B66" s="17" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C66" s="17" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D66" s="18" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
@@ -5733,26 +5733,26 @@
         <v>150</v>
       </c>
       <c r="H66" s="19" t="n">
-        <v>21.33333333333334</v>
+        <v>25.33333333333334</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
         <is>
-          <t>Chandrala B.O</t>
+          <t>Billapadu</t>
         </is>
       </c>
       <c r="B67" s="17" t="n">
-        <v>170</v>
+        <v>53</v>
       </c>
       <c r="C67" s="17" t="n">
-        <v>138</v>
+        <v>19</v>
       </c>
       <c r="D67" s="18" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
@@ -5766,10 +5766,10 @@
         <v>150</v>
       </c>
       <c r="H67" s="19" t="n">
-        <v>21.33333333333334</v>
+        <v>22.66666666666666</v>
       </c>
       <c r="I67" s="11" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="68">
@@ -5779,13 +5779,13 @@
         </is>
       </c>
       <c r="B68" s="17" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C68" s="17" t="n">
         <v>50</v>
       </c>
       <c r="D68" s="18" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
@@ -5799,26 +5799,26 @@
         <v>150</v>
       </c>
       <c r="H68" s="19" t="n">
-        <v>20.66666666666667</v>
+        <v>22</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>Vempadu B.O</t>
+          <t>Lingala B.O</t>
         </is>
       </c>
       <c r="B69" s="17" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C69" s="17" t="n">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="D69" s="18" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
@@ -5832,10 +5832,10 @@
         <v>150</v>
       </c>
       <c r="H69" s="19" t="n">
-        <v>18.66666666666667</v>
+        <v>21.33333333333334</v>
       </c>
       <c r="I69" s="11" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="70">
@@ -5947,10 +5947,10 @@
         <v>6</v>
       </c>
       <c r="C73" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D73" s="18" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
@@ -5964,10 +5964,10 @@
         <v>150</v>
       </c>
       <c r="H73" s="19" t="n">
-        <v>-3.333333333333333</v>
+        <v>-4.666666666666667</v>
       </c>
       <c r="I73" s="11" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -6051,13 +6051,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         <v>300</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>125.6666666666667</v>
+        <v>125.3333333333333</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -6084,13 +6084,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>56</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
         <v>300</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>117.3333333333333</v>
+        <v>117.6666666666667</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0</v>
@@ -6117,13 +6117,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>68</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -6137,7 +6137,7 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>105.3333333333333</v>
+        <v>106</v>
       </c>
       <c r="I4" s="6" t="n">
         <v>0</v>
@@ -6146,17 +6146,17 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Moturu S.O</t>
+          <t>Rudrapaka S.O</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>355</v>
+        <v>328</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -6170,26 +6170,26 @@
         <v>300</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>99.33333333333333</v>
+        <v>97.66666666666667</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Rudrapaka S.O</t>
+          <t>Moturu S.O</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>328</v>
+        <v>356</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -6203,10 +6203,10 @@
         <v>300</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>97.66666666666667</v>
+        <v>97.33333333333334</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -6216,13 +6216,13 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>96</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
@@ -6236,10 +6236,10 @@
         <v>300</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>90.33333333333333</v>
+        <v>92.33333333333333</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -6249,13 +6249,13 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>538</v>
+        <v>561</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -6269,10 +6269,10 @@
         <v>300</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>83.66666666666667</v>
+        <v>88</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9">
@@ -6282,13 +6282,13 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>31</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
@@ -6302,10 +6302,10 @@
         <v>300</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>71.66666666666667</v>
+        <v>72</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10">
@@ -6381,13 +6381,13 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>396</v>
+        <v>405</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
@@ -6401,10 +6401,10 @@
         <v>300</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>53.33333333333334</v>
+        <v>55.33333333333334</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13">
@@ -6414,13 +6414,13 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>14</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
@@ -6434,10 +6434,10 @@
         <v>300</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>46</v>
+        <v>47.66666666666667</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14">
@@ -6447,13 +6447,13 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>62</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
@@ -6467,10 +6467,10 @@
         <v>300</v>
       </c>
       <c r="H14" s="19" t="n">
-        <v>38.66666666666666</v>
+        <v>39</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15">
@@ -6620,13 +6620,13 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1430</v>
+        <v>1457</v>
       </c>
       <c r="C2" s="13" t="n">
-        <v>918</v>
+        <v>947</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
@@ -6640,10 +6640,10 @@
         <v>1000</v>
       </c>
       <c r="H2" s="15" t="n">
-        <v>51.2</v>
+        <v>51</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>
@@ -6763,10 +6763,10 @@
         <v>239</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>150</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>130</v>
+        <v>123.3333333333333</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0</v>
@@ -6796,10 +6796,10 @@
         <v>253</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -6813,7 +6813,7 @@
         <v>150</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>128.6666666666667</v>
+        <v>115.3333333333333</v>
       </c>
       <c r="I4" s="6" t="n">
         <v>0</v>
@@ -6969,10 +6969,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2" s="18" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
@@ -6986,10 +6986,10 @@
         <v>150</v>
       </c>
       <c r="H2" s="19" t="n">
-        <v>-3.333333333333333</v>
+        <v>-4.666666666666667</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3">
@@ -7094,17 +7094,17 @@
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Vempadu B.O</t>
+          <t>Lingala B.O</t>
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
@@ -7118,10 +7118,10 @@
         <v>150</v>
       </c>
       <c r="H6" s="19" t="n">
-        <v>18.66666666666667</v>
+        <v>21.33333333333334</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -7205,13 +7205,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -7225,7 +7225,7 @@
         <v>300</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>125.6666666666667</v>
+        <v>125.3333333333333</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -7238,13 +7238,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>56</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -7258,7 +7258,7 @@
         <v>300</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>117.3333333333333</v>
+        <v>117.6666666666667</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0</v>
@@ -7271,13 +7271,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>68</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -7291,7 +7291,7 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>105.3333333333333</v>
+        <v>106</v>
       </c>
       <c r="I4" s="6" t="n">
         <v>0</v>
@@ -7444,13 +7444,13 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C4" s="17" t="n">
         <v>62</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
@@ -7464,10 +7464,10 @@
         <v>300</v>
       </c>
       <c r="H4" s="19" t="n">
-        <v>38.66666666666666</v>
+        <v>39</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7568,7 +7568,7 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>15966</v>
+        <v>16234</v>
       </c>
     </row>
     <row r="8">
@@ -7578,7 +7578,7 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>5602</v>
+        <v>5815</v>
       </c>
     </row>
     <row r="9">
@@ -7588,7 +7588,7 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>10364</v>
+        <v>10419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>